<commit_message>
Main board BOM edits
</commit_message>
<xml_diff>
--- a/01-main_board/main_board_v3/DigikeyOrdering/BOM-main_board_v3.xlsx
+++ b/01-main_board/main_board_v3/DigikeyOrdering/BOM-main_board_v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emma/Documents/JHU/22xt_kicad/01-main_board/main_board_v3/DigikeyOrdering/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{03246B71-3A5E-C84E-B0FE-E9A753A9678A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{34C7EF8D-1F13-8045-BD7D-DE6C37C5C6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35840" yWindow="0" windowWidth="34360" windowHeight="28800" xr2:uid="{E864DD15-E767-464B-8250-0CE0FF16D1D0}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{E864DD15-E767-464B-8250-0CE0FF16D1D0}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM-main_board_v3" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="194">
   <si>
     <t>Comment</t>
   </si>
@@ -590,6 +590,18 @@
   </si>
   <si>
     <t>but 0201</t>
+  </si>
+  <si>
+    <t>not on mouser</t>
+  </si>
+  <si>
+    <t>XXXX</t>
+  </si>
+  <si>
+    <t>a billion</t>
+  </si>
+  <si>
+    <t>XX</t>
   </si>
 </sst>
 </file>
@@ -1971,7 +1983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>43</v>
       </c>
@@ -1986,7 +1998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>43</v>
       </c>
@@ -2001,7 +2013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>43</v>
       </c>
@@ -2016,7 +2028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>43</v>
       </c>
@@ -2031,7 +2043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>43</v>
       </c>
@@ -2046,7 +2058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>145</v>
       </c>
@@ -2063,7 +2075,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>145</v>
       </c>
@@ -2080,7 +2092,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>67</v>
       </c>
@@ -2097,7 +2109,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>43</v>
       </c>
@@ -2112,7 +2124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>43</v>
       </c>
@@ -2127,7 +2139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>125</v>
       </c>
@@ -2140,8 +2152,11 @@
       <c r="E43">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>150</v>
       </c>
@@ -2154,8 +2169,11 @@
       <c r="E44">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>117</v>
       </c>
@@ -2168,8 +2186,11 @@
       <c r="E45">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>38</v>
       </c>
@@ -2182,8 +2203,14 @@
       <c r="E46">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="I46" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>133</v>
       </c>
@@ -2196,8 +2223,14 @@
       <c r="E47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G47">
+        <v>3</v>
+      </c>
+      <c r="H47">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>56</v>
       </c>
@@ -2210,8 +2243,11 @@
       <c r="E48">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G48">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>34</v>
       </c>
@@ -2231,7 +2267,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -2248,7 +2284,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>47</v>
       </c>
@@ -2264,8 +2300,11 @@
       <c r="G51">
         <v>2</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H51">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -2282,7 +2321,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>86</v>
       </c>
@@ -2295,8 +2334,11 @@
       <c r="E53">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>81</v>
       </c>
@@ -2309,8 +2351,11 @@
       <c r="E54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>99</v>
       </c>
@@ -2323,8 +2368,14 @@
       <c r="E55">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G55">
+        <v>1</v>
+      </c>
+      <c r="H55">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>89</v>
       </c>
@@ -2338,10 +2389,10 @@
         <v>1</v>
       </c>
       <c r="G56">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>16</v>
       </c>
@@ -2358,7 +2409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>69</v>
       </c>
@@ -2371,8 +2422,11 @@
       <c r="E58">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H58" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>9</v>
       </c>
@@ -2389,7 +2443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>47</v>
       </c>
@@ -2403,7 +2457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>110</v>
       </c>
@@ -2417,7 +2471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>110</v>
       </c>
@@ -2431,7 +2485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>110</v>
       </c>
@@ -2445,7 +2499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>110</v>
       </c>
@@ -2481,7 +2535,7 @@
         <v>168</v>
       </c>
       <c r="C66" t="s">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -2596,6 +2650,9 @@
       <c r="E73">
         <v>1</v>
       </c>
+      <c r="G73">
+        <v>10</v>
+      </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
@@ -2610,6 +2667,9 @@
       <c r="E74">
         <v>1</v>
       </c>
+      <c r="G74">
+        <v>10</v>
+      </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
@@ -2639,7 +2699,7 @@
         <v>1</v>
       </c>
       <c r="G76">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
@@ -2917,6 +2977,9 @@
       <c r="E94">
         <v>1</v>
       </c>
+      <c r="G94">
+        <v>10</v>
+      </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95">
@@ -2949,10 +3012,10 @@
         <v>1</v>
       </c>
       <c r="G96">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>13</v>
       </c>
@@ -2969,7 +3032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>108</v>
       </c>
@@ -2986,7 +3049,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>108</v>
       </c>
@@ -3003,7 +3066,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>108</v>
       </c>
@@ -3020,7 +3083,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>159</v>
       </c>
@@ -3034,10 +3097,10 @@
         <v>1</v>
       </c>
       <c r="G101">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>115</v>
       </c>
@@ -3054,7 +3117,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>62</v>
       </c>
@@ -3068,7 +3131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>749013011</v>
       </c>
@@ -3085,7 +3148,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>105</v>
       </c>
@@ -3098,8 +3161,14 @@
       <c r="E105">
         <v>1</v>
       </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G105">
+        <v>1</v>
+      </c>
+      <c r="H105">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>154</v>
       </c>
@@ -3116,7 +3185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>122</v>
       </c>
@@ -3129,8 +3198,11 @@
       <c r="E107">
         <v>1</v>
       </c>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G107" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>77</v>
       </c>
@@ -3144,10 +3216,10 @@
         <v>1</v>
       </c>
       <c r="G108">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>96</v>
       </c>
@@ -3159,6 +3231,12 @@
       </c>
       <c r="E109">
         <v>1</v>
+      </c>
+      <c r="G109">
+        <v>1</v>
+      </c>
+      <c r="H109" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>